<commit_message>
fix(payroll): keep workbook source notes out of imported categories
</commit_message>
<xml_diff>
--- a/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
+++ b/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="R480793e5d42e4a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Re9635f5662cd467b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="R783d2aa6cb3745f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R1d24b1a4ea2345ca"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="PayrollHeader">'Payroll'!A1:Y1</x:definedName>

</xml_diff>

<commit_message>
fix(payroll): use Singapore formulas supported by the deployed engine
</commit_message>
<xml_diff>
--- a/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
+++ b/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="R783d2aa6cb3745f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R1d24b1a4ea2345ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="R7552b577a2e24912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R1b286ea4e486405a"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="PayrollHeader">'Payroll'!A1:Y1</x:definedName>

</xml_diff>

<commit_message>
feat(payroll): finish Singapore review configuration and import handover
</commit_message>
<xml_diff>
--- a/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
+++ b/outputs/sg-payroll-20261014/Rize_Singapore_Monthly_Inputs.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="R7552b577a2e24912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R1b286ea4e486405a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll" sheetId="1" r:id="Rbc64c1c01b874116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R98aa723c3b7441d8"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="PayrollHeader">'Payroll'!A1:Y1</x:definedName>
@@ -8657,7 +8657,7 @@
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>In Pay Run, select the Singapore configuration and month, upload this file at Pay data, then review employee matching and results.</x:v>
+        <x:v>After configuration activation, select the Singapore payroll and month in Pay Run. Upload this file at Pay data and review matches and results.</x:v>
       </x:c>
       <x:c r="B11" s="2"/>
       <x:c r="C11" s="2"/>
@@ -8666,7 +8666,7 @@
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>The app calculates SDL and outputs. Do not add formulas, statutory tables, annual CTC or take-home-pay columns to this upload file.</x:v>
+        <x:v>Choose This run only for monthly values. Choose Update Payobook when approved employee, contract or bank changes should be saved.</x:v>
       </x:c>
       <x:c r="B12" s="2"/>
       <x:c r="C12" s="2"/>
@@ -8675,7 +8675,7 @@
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>Sum all employee SDL amounts and round the employer remittance down to whole dollars. Individual payroll cost retains exact SDL.</x:v>
+        <x:v>The app calculates SDL and outputs. Do not add formulas, statutory tables, annual CTC or take-home-pay columns to this upload file.</x:v>
       </x:c>
       <x:c r="B13" s="2"/>
       <x:c r="C13" s="2"/>
@@ -8684,7 +8684,7 @@
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>This monthly template does not calculate FnF, IR21 withholding, bonus CPF/AW limits or automated citizen/PR contribution rates.</x:v>
+        <x:v>Sum all employee SDL amounts and round the employer remittance down to whole dollars. Individual payroll cost retains exact SDL.</x:v>
       </x:c>
       <x:c r="B14" s="2"/>
       <x:c r="C14" s="2"/>
@@ -8692,7 +8692,9 @@
       <x:c r="E14" s="2"/>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="2"/>
+      <x:c r="A15" s="2" t="str">
+        <x:v>This monthly template does not calculate FnF, IR21 withholding, bonus CPF/AW limits or automated citizen/PR contribution rates.</x:v>
+      </x:c>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -9230,6 +9232,7 @@
     <x:mergeCell ref="A12:E12"/>
     <x:mergeCell ref="A13:E13"/>
     <x:mergeCell ref="A14:E14"/>
+    <x:mergeCell ref="A15:E15"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>